<commit_message>
Clean project and dataset
</commit_message>
<xml_diff>
--- a/DATA/Export 2007-2024.xlsx
+++ b/DATA/Export 2007-2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noxra\KMUTNB_internship\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8A4B9E-FE4E-4D25-B597-9E0B4AFCBBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F422429-BE09-4B0B-80D3-2C77F4C426E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Year (พ.ศ.)</t>
   </si>
@@ -211,579 +211,6 @@
   </si>
   <si>
     <t>Grand Total Value (Million Baht)</t>
-  </si>
-  <si>
-    <t>34.750</t>
-  </si>
-  <si>
-    <t>34.025</t>
-  </si>
-  <si>
-    <t>32.325</t>
-  </si>
-  <si>
-    <t>32.850</t>
-  </si>
-  <si>
-    <t>32.900</t>
-  </si>
-  <si>
-    <t>31.700</t>
-  </si>
-  <si>
-    <t>29.950</t>
-  </si>
-  <si>
-    <t>32.535</t>
-  </si>
-  <si>
-    <t>31.900</t>
-  </si>
-  <si>
-    <t>31.675</t>
-  </si>
-  <si>
-    <t>30.700</t>
-  </si>
-  <si>
-    <t>30.050</t>
-  </si>
-  <si>
-    <t>31.300</t>
-  </si>
-  <si>
-    <t>31.075</t>
-  </si>
-  <si>
-    <t>31.470</t>
-  </si>
-  <si>
-    <t>31.655</t>
-  </si>
-  <si>
-    <t>32.489</t>
-  </si>
-  <si>
-    <t>33.430</t>
-  </si>
-  <si>
-    <t>33.520</t>
-  </si>
-  <si>
-    <t>34.225</t>
-  </si>
-  <si>
-    <t>33.855</t>
-  </si>
-  <si>
-    <t>35.050</t>
-  </si>
-  <si>
-    <t>35.470</t>
-  </si>
-  <si>
-    <t>34.785</t>
-  </si>
-  <si>
-    <t>34.975</t>
-  </si>
-  <si>
-    <t>36.190</t>
-  </si>
-  <si>
-    <t>35.495</t>
-  </si>
-  <si>
-    <t>35.280</t>
-  </si>
-  <si>
-    <t>34.310</t>
-  </si>
-  <si>
-    <t>34.060</t>
-  </si>
-  <si>
-    <t>34.020</t>
-  </si>
-  <si>
-    <t>33.440</t>
-  </si>
-  <si>
-    <t>33.455</t>
-  </si>
-  <si>
-    <t>33.235</t>
-  </si>
-  <si>
-    <t>33.360</t>
-  </si>
-  <si>
-    <t>33.175</t>
-  </si>
-  <si>
-    <t>33.055</t>
-  </si>
-  <si>
-    <t>32.350</t>
-  </si>
-  <si>
-    <t>32.345</t>
-  </si>
-  <si>
-    <t>32.530</t>
-  </si>
-  <si>
-    <t>32.415</t>
-  </si>
-  <si>
-    <t>32.240</t>
-  </si>
-  <si>
-    <t>31.270</t>
-  </si>
-  <si>
-    <t>30.345</t>
-  </si>
-  <si>
-    <t>29.940</t>
-  </si>
-  <si>
-    <t>30.185</t>
-  </si>
-  <si>
-    <t>30.065</t>
-  </si>
-  <si>
-    <t>30.905</t>
-  </si>
-  <si>
-    <t>30.595</t>
-  </si>
-  <si>
-    <t>30.255</t>
-  </si>
-  <si>
-    <t>29.850</t>
-  </si>
-  <si>
-    <t>30.300</t>
-  </si>
-  <si>
-    <t>29.750</t>
-  </si>
-  <si>
-    <t>29.930</t>
-  </si>
-  <si>
-    <t>31.170</t>
-  </si>
-  <si>
-    <t>30.840</t>
-  </si>
-  <si>
-    <t>31.520</t>
-  </si>
-  <si>
-    <t>30.970</t>
-  </si>
-  <si>
-    <t>30.440</t>
-  </si>
-  <si>
-    <t>30.830</t>
-  </si>
-  <si>
-    <t>30.720</t>
-  </si>
-  <si>
-    <t>31.840</t>
-  </si>
-  <si>
-    <t>31.540</t>
-  </si>
-  <si>
-    <t>31.500</t>
-  </si>
-  <si>
-    <t>31.320</t>
-  </si>
-  <si>
-    <t>30.810</t>
-  </si>
-  <si>
-    <t>30.690</t>
-  </si>
-  <si>
-    <t>30.580</t>
-  </si>
-  <si>
-    <t>29.800</t>
-  </si>
-  <si>
-    <t>29.760</t>
-  </si>
-  <si>
-    <t>29.280</t>
-  </si>
-  <si>
-    <t>29.260</t>
-  </si>
-  <si>
-    <t>30.410</t>
-  </si>
-  <si>
-    <t>31.120</t>
-  </si>
-  <si>
-    <t>31.340</t>
-  </si>
-  <si>
-    <t>32.130</t>
-  </si>
-  <si>
-    <t>31.210</t>
-  </si>
-  <si>
-    <t>31.140</t>
-  </si>
-  <si>
-    <t>32.030</t>
-  </si>
-  <si>
-    <t>32.680</t>
-  </si>
-  <si>
-    <t>33.010</t>
-  </si>
-  <si>
-    <t>32.520</t>
-  </si>
-  <si>
-    <t>32.390</t>
-  </si>
-  <si>
-    <t>32.340</t>
-  </si>
-  <si>
-    <t>32.810</t>
-  </si>
-  <si>
-    <t>32.410</t>
-  </si>
-  <si>
-    <t>32.180</t>
-  </si>
-  <si>
-    <t>31.920</t>
-  </si>
-  <si>
-    <t>32.420</t>
-  </si>
-  <si>
-    <t>32.580</t>
-  </si>
-  <si>
-    <t>32.720</t>
-  </si>
-  <si>
-    <t>33.690</t>
-  </si>
-  <si>
-    <t>33.790</t>
-  </si>
-  <si>
-    <t>34.990</t>
-  </si>
-  <si>
-    <t>35.820</t>
-  </si>
-  <si>
-    <t>36.360</t>
-  </si>
-  <si>
-    <t>35.590</t>
-  </si>
-  <si>
-    <t>35.790</t>
-  </si>
-  <si>
-    <t>36.020</t>
-  </si>
-  <si>
-    <t>35.710</t>
-  </si>
-  <si>
-    <t>35.610</t>
-  </si>
-  <si>
-    <t>35.100</t>
-  </si>
-  <si>
-    <t>34.890</t>
-  </si>
-  <si>
-    <t>35.760</t>
-  </si>
-  <si>
-    <t>34.760</t>
-  </si>
-  <si>
-    <t>34.620</t>
-  </si>
-  <si>
-    <t>34.580</t>
-  </si>
-  <si>
-    <t>35.020</t>
-  </si>
-  <si>
-    <t>35.690</t>
-  </si>
-  <si>
-    <t>35.840</t>
-  </si>
-  <si>
-    <t>35.080</t>
-  </si>
-  <si>
-    <t>34.930</t>
-  </si>
-  <si>
-    <t>34.340</t>
-  </si>
-  <si>
-    <t>34.030</t>
-  </si>
-  <si>
-    <t>33.920</t>
-  </si>
-  <si>
-    <t>33.290</t>
-  </si>
-  <si>
-    <t>33.170</t>
-  </si>
-  <si>
-    <t>33.320</t>
-  </si>
-  <si>
-    <t>33.220</t>
-  </si>
-  <si>
-    <t>32.640</t>
-  </si>
-  <si>
-    <t>32.550</t>
-  </si>
-  <si>
-    <t>31.480</t>
-  </si>
-  <si>
-    <t>32.050</t>
-  </si>
-  <si>
-    <t>33.020</t>
-  </si>
-  <si>
-    <t>33.190</t>
-  </si>
-  <si>
-    <t>32.750</t>
-  </si>
-  <si>
-    <t>32.320</t>
-  </si>
-  <si>
-    <t>33.110</t>
-  </si>
-  <si>
-    <t>32.960</t>
-  </si>
-  <si>
-    <t>32.330</t>
-  </si>
-  <si>
-    <t>31.200</t>
-  </si>
-  <si>
-    <t>31.570</t>
-  </si>
-  <si>
-    <t>31.720</t>
-  </si>
-  <si>
-    <t>31.890</t>
-  </si>
-  <si>
-    <t>30.680</t>
-  </si>
-  <si>
-    <t>30.600</t>
-  </si>
-  <si>
-    <t>30.590</t>
-  </si>
-  <si>
-    <t>30.180</t>
-  </si>
-  <si>
-    <t>30.190</t>
-  </si>
-  <si>
-    <t>31.510</t>
-  </si>
-  <si>
-    <t>32.740</t>
-  </si>
-  <si>
-    <t>32.450</t>
-  </si>
-  <si>
-    <t>31.810</t>
-  </si>
-  <si>
-    <t>30.900</t>
-  </si>
-  <si>
-    <t>31.250</t>
-  </si>
-  <si>
-    <t>31.070</t>
-  </si>
-  <si>
-    <t>31.600</t>
-  </si>
-  <si>
-    <t>30.280</t>
-  </si>
-  <si>
-    <t>30.040</t>
-  </si>
-  <si>
-    <t>29.860</t>
-  </si>
-  <si>
-    <t>30.470</t>
-  </si>
-  <si>
-    <t>31.240</t>
-  </si>
-  <si>
-    <t>31.190</t>
-  </si>
-  <si>
-    <t>32.020</t>
-  </si>
-  <si>
-    <t>32.890</t>
-  </si>
-  <si>
-    <t>32.220</t>
-  </si>
-  <si>
-    <t>33.670</t>
-  </si>
-  <si>
-    <t>33.710</t>
-  </si>
-  <si>
-    <t>33.230</t>
-  </si>
-  <si>
-    <t>32.670</t>
-  </si>
-  <si>
-    <t>33.280</t>
-  </si>
-  <si>
-    <t>34.240</t>
-  </si>
-  <si>
-    <t>34.300</t>
-  </si>
-  <si>
-    <t>35.300</t>
-  </si>
-  <si>
-    <t>36.290</t>
-  </si>
-  <si>
-    <t>36.520</t>
-  </si>
-  <si>
-    <t>37.770</t>
-  </si>
-  <si>
-    <t>38.050</t>
-  </si>
-  <si>
-    <t>35.110</t>
-  </si>
-  <si>
-    <t>34.610</t>
-  </si>
-  <si>
-    <t>32.840</t>
-  </si>
-  <si>
-    <t>35.220</t>
-  </si>
-  <si>
-    <t>34.160</t>
-  </si>
-  <si>
-    <t>34.120</t>
-  </si>
-  <si>
-    <t>34.640</t>
-  </si>
-  <si>
-    <t>35.270</t>
-  </si>
-  <si>
-    <t>34.210</t>
-  </si>
-  <si>
-    <t>34.980</t>
-  </si>
-  <si>
-    <t>36.510</t>
-  </si>
-  <si>
-    <t>36.140</t>
-  </si>
-  <si>
-    <t>35.310</t>
-  </si>
-  <si>
-    <t>34.350</t>
-  </si>
-  <si>
-    <t>35.530</t>
-  </si>
-  <si>
-    <t>35.880</t>
-  </si>
-  <si>
-    <t>36.370</t>
-  </si>
-  <si>
-    <t>37.180</t>
-  </si>
-  <si>
-    <t>36.770</t>
-  </si>
-  <si>
-    <t>36.760</t>
-  </si>
-  <si>
-    <t>34.270</t>
-  </si>
-  <si>
-    <t>34.260</t>
-  </si>
-  <si>
-    <t>Price baht to usd</t>
   </si>
 </sst>
 </file>
@@ -2509,13 +1936,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BK217"/>
+  <dimension ref="A1:BJ217"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="63" max="63" width="7.5546875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:63" ht="211.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:62" ht="211.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="230" t="s">
         <v>0</v>
       </c>
@@ -2702,11 +2126,8 @@
       <c r="BJ1" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" t="s">
-        <v>252</v>
-      </c>
     </row>
-    <row r="2" spans="1:63" ht="21.6" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:62" ht="21.6" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="233">
         <v>2550</v>
       </c>
@@ -2889,11 +2310,8 @@
       <c r="BJ2" s="35">
         <v>14562.65</v>
       </c>
-      <c r="BK2" t="s">
-        <v>62</v>
-      </c>
     </row>
-    <row r="3" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A3" s="233">
         <v>2550</v>
       </c>
@@ -3076,11 +2494,8 @@
       <c r="BJ3" s="45">
         <v>15295.19</v>
       </c>
-      <c r="BK3" t="s">
-        <v>63</v>
-      </c>
     </row>
-    <row r="4" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A4" s="233">
         <v>2550</v>
       </c>
@@ -3263,11 +2678,8 @@
       <c r="BJ4" s="45">
         <v>17811.330000000002</v>
       </c>
-      <c r="BK4" t="s">
-        <v>64</v>
-      </c>
     </row>
-    <row r="5" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A5" s="233">
         <v>2550</v>
       </c>
@@ -3450,11 +2862,8 @@
       <c r="BJ5" s="45">
         <v>14369.74</v>
       </c>
-      <c r="BK5" t="s">
-        <v>65</v>
-      </c>
     </row>
-    <row r="6" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="233">
         <v>2550</v>
       </c>
@@ -3637,11 +3046,8 @@
       <c r="BJ6" s="45">
         <v>17047.87</v>
       </c>
-      <c r="BK6" t="s">
-        <v>66</v>
-      </c>
     </row>
-    <row r="7" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A7" s="233">
         <v>2550</v>
       </c>
@@ -3824,11 +3230,8 @@
       <c r="BJ7" s="45">
         <v>16817.580000000002</v>
       </c>
-      <c r="BK7" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="8" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A8" s="233">
         <v>2550</v>
       </c>
@@ -4011,11 +3414,8 @@
       <c r="BJ8" s="45">
         <v>16511.490000000002</v>
       </c>
-      <c r="BK8" t="s">
-        <v>68</v>
-      </c>
     </row>
-    <row r="9" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="233">
         <v>2550</v>
       </c>
@@ -4198,11 +3598,8 @@
       <c r="BJ9" s="45">
         <v>18631.689999999999</v>
       </c>
-      <c r="BK9" t="s">
-        <v>69</v>
-      </c>
     </row>
-    <row r="10" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="233">
         <v>2550</v>
       </c>
@@ -4385,11 +3782,8 @@
       <c r="BJ10" s="45">
         <v>18730.71</v>
       </c>
-      <c r="BK10" t="s">
-        <v>70</v>
-      </c>
     </row>
-    <row r="11" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="233">
         <v>2550</v>
       </c>
@@ -4572,11 +3966,8 @@
       <c r="BJ11" s="45">
         <v>19519.5</v>
       </c>
-      <c r="BK11" t="s">
-        <v>71</v>
-      </c>
     </row>
-    <row r="12" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="233">
         <v>2550</v>
       </c>
@@ -4759,11 +4150,8 @@
       <c r="BJ12" s="45">
         <v>19822.48</v>
       </c>
-      <c r="BK12" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="13" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="233">
         <v>2550</v>
       </c>
@@ -4946,11 +4334,8 @@
       <c r="BJ13" s="45">
         <v>16746.47</v>
       </c>
-      <c r="BK13" t="s">
-        <v>73</v>
-      </c>
     </row>
-    <row r="14" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="235">
         <v>2551</v>
       </c>
@@ -5133,11 +4518,8 @@
       <c r="BJ14" s="58">
         <v>16057.08</v>
       </c>
-      <c r="BK14" t="s">
-        <v>74</v>
-      </c>
     </row>
-    <row r="15" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="235">
         <v>2551</v>
       </c>
@@ -5320,11 +4702,8 @@
       <c r="BJ15" s="58">
         <v>15277.18</v>
       </c>
-      <c r="BK15" t="s">
-        <v>75</v>
-      </c>
     </row>
-    <row r="16" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="235">
         <v>2551</v>
       </c>
@@ -5507,11 +4886,8 @@
       <c r="BJ16" s="58">
         <v>16991.54</v>
       </c>
-      <c r="BK16" t="s">
-        <v>76</v>
-      </c>
     </row>
-    <row r="17" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="235">
         <v>2551</v>
       </c>
@@ -5694,11 +5070,8 @@
       <c r="BJ17" s="58">
         <v>16436.21</v>
       </c>
-      <c r="BK17" t="s">
-        <v>77</v>
-      </c>
     </row>
-    <row r="18" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="235">
         <v>2551</v>
       </c>
@@ -5881,11 +5254,8 @@
       <c r="BJ18" s="58">
         <v>18279.72</v>
       </c>
-      <c r="BK18" t="s">
-        <v>78</v>
-      </c>
     </row>
-    <row r="19" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="235">
         <v>2551</v>
       </c>
@@ -6068,11 +5438,8 @@
       <c r="BJ19" s="58">
         <v>18215.37</v>
       </c>
-      <c r="BK19" t="s">
-        <v>79</v>
-      </c>
     </row>
-    <row r="20" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="235">
         <v>2551</v>
       </c>
@@ -6255,11 +5622,8 @@
       <c r="BJ20" s="58">
         <v>21335.82</v>
       </c>
-      <c r="BK20" t="s">
-        <v>80</v>
-      </c>
     </row>
-    <row r="21" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="235">
         <v>2551</v>
       </c>
@@ -6442,11 +5806,8 @@
       <c r="BJ21" s="58">
         <v>21546.91</v>
       </c>
-      <c r="BK21" t="s">
-        <v>81</v>
-      </c>
     </row>
-    <row r="22" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="235">
         <v>2551</v>
       </c>
@@ -6629,11 +5990,8 @@
       <c r="BJ22" s="58">
         <v>21304.31</v>
       </c>
-      <c r="BK22" t="s">
-        <v>82</v>
-      </c>
     </row>
-    <row r="23" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="235">
         <v>2551</v>
       </c>
@@ -6816,11 +6174,8 @@
       <c r="BJ23" s="58">
         <v>23647.56</v>
       </c>
-      <c r="BK23" t="s">
-        <v>83</v>
-      </c>
     </row>
-    <row r="24" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="235">
         <v>2551</v>
       </c>
@@ -7003,11 +6358,8 @@
       <c r="BJ24" s="58">
         <v>20792.3</v>
       </c>
-      <c r="BK24" t="s">
-        <v>84</v>
-      </c>
     </row>
-    <row r="25" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="235">
         <v>2551</v>
       </c>
@@ -7190,11 +6542,8 @@
       <c r="BJ25" s="58">
         <v>18333.650000000001</v>
       </c>
-      <c r="BK25" t="s">
-        <v>85</v>
-      </c>
     </row>
-    <row r="26" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="237">
         <v>2552</v>
       </c>
@@ -7377,11 +6726,8 @@
       <c r="BJ26" s="71">
         <v>15085.79</v>
       </c>
-      <c r="BK26" t="s">
-        <v>86</v>
-      </c>
     </row>
-    <row r="27" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="237">
         <v>2552</v>
       </c>
@@ -7564,11 +6910,8 @@
       <c r="BJ27" s="71">
         <v>15226.44</v>
       </c>
-      <c r="BK27" t="s">
-        <v>87</v>
-      </c>
     </row>
-    <row r="28" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="237">
         <v>2552</v>
       </c>
@@ -7751,11 +7094,8 @@
       <c r="BJ28" s="71">
         <v>16837.8</v>
       </c>
-      <c r="BK28" t="s">
-        <v>88</v>
-      </c>
     </row>
-    <row r="29" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="237">
         <v>2552</v>
       </c>
@@ -7938,11 +7278,8 @@
       <c r="BJ29" s="71">
         <v>16995.099999999999</v>
       </c>
-      <c r="BK29" t="s">
-        <v>89</v>
-      </c>
     </row>
-    <row r="30" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="237">
         <v>2552</v>
       </c>
@@ -8125,11 +7462,8 @@
       <c r="BJ30" s="71">
         <v>18387.93</v>
       </c>
-      <c r="BK30" t="s">
-        <v>90</v>
-      </c>
     </row>
-    <row r="31" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="237">
         <v>2552</v>
       </c>
@@ -8312,11 +7646,8 @@
       <c r="BJ31" s="71">
         <v>18945.830000000002</v>
       </c>
-      <c r="BK31" t="s">
-        <v>91</v>
-      </c>
     </row>
-    <row r="32" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="237">
         <v>2552</v>
       </c>
@@ -8499,11 +7830,8 @@
       <c r="BJ32" s="71">
         <v>20722.89</v>
       </c>
-      <c r="BK32" t="s">
-        <v>63</v>
-      </c>
     </row>
-    <row r="33" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="237">
         <v>2552</v>
       </c>
@@ -8686,11 +8014,8 @@
       <c r="BJ33" s="71">
         <v>19484.169999999998</v>
       </c>
-      <c r="BK33" t="s">
-        <v>92</v>
-      </c>
     </row>
-    <row r="34" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="237">
         <v>2552</v>
       </c>
@@ -8873,11 +8198,8 @@
       <c r="BJ34" s="71">
         <v>21099.3</v>
       </c>
-      <c r="BK34" t="s">
-        <v>93</v>
-      </c>
     </row>
-    <row r="35" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="237">
         <v>2552</v>
       </c>
@@ -9060,11 +8382,8 @@
       <c r="BJ35" s="71">
         <v>22469.599999999999</v>
       </c>
-      <c r="BK35" t="s">
-        <v>94</v>
-      </c>
     </row>
-    <row r="36" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="237">
         <v>2552</v>
       </c>
@@ -9247,11 +8566,8 @@
       <c r="BJ36" s="71">
         <v>19982.599999999999</v>
       </c>
-      <c r="BK36" t="s">
-        <v>95</v>
-      </c>
     </row>
-    <row r="37" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="237">
         <v>2552</v>
       </c>
@@ -9434,11 +8750,8 @@
       <c r="BJ37" s="71">
         <v>19275.16</v>
       </c>
-      <c r="BK37" t="s">
-        <v>96</v>
-      </c>
     </row>
-    <row r="38" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="239">
         <v>2553</v>
       </c>
@@ -9621,11 +8934,8 @@
       <c r="BJ38" s="83">
         <v>16952.330000000002</v>
       </c>
-      <c r="BK38" t="s">
-        <v>97</v>
-      </c>
     </row>
-    <row r="39" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="239">
         <v>2553</v>
       </c>
@@ -9808,11 +9118,8 @@
       <c r="BJ39" s="83">
         <v>16616.150000000001</v>
       </c>
-      <c r="BK39" t="s">
-        <v>98</v>
-      </c>
     </row>
-    <row r="40" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="239">
         <v>2553</v>
       </c>
@@ -9995,11 +9302,8 @@
       <c r="BJ40" s="83">
         <v>19955.169999999998</v>
       </c>
-      <c r="BK40" t="s">
-        <v>99</v>
-      </c>
     </row>
-    <row r="41" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="239">
         <v>2553</v>
       </c>
@@ -10182,11 +9486,8 @@
       <c r="BJ41" s="83">
         <v>15998.3</v>
       </c>
-      <c r="BK41" t="s">
-        <v>100</v>
-      </c>
     </row>
-    <row r="42" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="239">
         <v>2553</v>
       </c>
@@ -10369,11 +9670,8 @@
       <c r="BJ42" s="83">
         <v>18623.64</v>
       </c>
-      <c r="BK42" t="s">
-        <v>101</v>
-      </c>
     </row>
-    <row r="43" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="239">
         <v>2553</v>
       </c>
@@ -10556,11 +9854,8 @@
       <c r="BJ43" s="83">
         <v>22790.23</v>
       </c>
-      <c r="BK43" t="s">
-        <v>102</v>
-      </c>
     </row>
-    <row r="44" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="239">
         <v>2553</v>
       </c>
@@ -10743,11 +10038,8 @@
       <c r="BJ44" s="83">
         <v>20850.78</v>
       </c>
-      <c r="BK44" t="s">
-        <v>103</v>
-      </c>
     </row>
-    <row r="45" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A45" s="239">
         <v>2553</v>
       </c>
@@ -10930,11 +10222,8 @@
       <c r="BJ45" s="83">
         <v>20175.84</v>
       </c>
-      <c r="BK45" t="s">
-        <v>104</v>
-      </c>
     </row>
-    <row r="46" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A46" s="239">
         <v>2553</v>
       </c>
@@ -11117,11 +10406,8 @@
       <c r="BJ46" s="83">
         <v>21309.7</v>
       </c>
-      <c r="BK46" t="s">
-        <v>105</v>
-      </c>
     </row>
-    <row r="47" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A47" s="239">
         <v>2553</v>
       </c>
@@ -11304,11 +10590,8 @@
       <c r="BJ47" s="83">
         <v>21922.23</v>
       </c>
-      <c r="BK47" t="s">
-        <v>106</v>
-      </c>
     </row>
-    <row r="48" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A48" s="239">
         <v>2553</v>
       </c>
@@ -11491,11 +10774,8 @@
       <c r="BJ48" s="83">
         <v>21191.200000000001</v>
       </c>
-      <c r="BK48" t="s">
-        <v>107</v>
-      </c>
     </row>
-    <row r="49" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A49" s="239">
         <v>2553</v>
       </c>
@@ -11678,11 +10958,8 @@
       <c r="BJ49" s="83">
         <v>20516.57</v>
       </c>
-      <c r="BK49" t="s">
-        <v>108</v>
-      </c>
     </row>
-    <row r="50" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A50" s="241">
         <v>2554</v>
       </c>
@@ -11865,11 +11142,8 @@
       <c r="BJ50" s="96">
         <v>16954.03</v>
       </c>
-      <c r="BK50" t="s">
-        <v>109</v>
-      </c>
     </row>
-    <row r="51" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A51" s="241">
         <v>2554</v>
       </c>
@@ -12052,11 +11326,8 @@
       <c r="BJ51" s="96">
         <v>17437.72</v>
       </c>
-      <c r="BK51" t="s">
-        <v>110</v>
-      </c>
     </row>
-    <row r="52" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A52" s="241">
         <v>2554</v>
       </c>
@@ -12239,11 +11510,8 @@
       <c r="BJ52" s="96">
         <v>21532.959999999999</v>
       </c>
-      <c r="BK52" t="s">
-        <v>111</v>
-      </c>
     </row>
-    <row r="53" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A53" s="241">
         <v>2554</v>
       </c>
@@ -12426,11 +11694,8 @@
       <c r="BJ53" s="96">
         <v>17814.04</v>
       </c>
-      <c r="BK53" t="s">
-        <v>112</v>
-      </c>
     </row>
-    <row r="54" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A54" s="241">
         <v>2554</v>
       </c>
@@ -12613,11 +11878,8 @@
       <c r="BJ54" s="96">
         <v>20535.39</v>
       </c>
-      <c r="BK54" t="s">
-        <v>113</v>
-      </c>
     </row>
-    <row r="55" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A55" s="241">
         <v>2554</v>
       </c>
@@ -12800,11 +12062,8 @@
       <c r="BJ55" s="96">
         <v>23011.09</v>
       </c>
-      <c r="BK55" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="56" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A56" s="241">
         <v>2554</v>
       </c>
@@ -12987,11 +12246,8 @@
       <c r="BJ56" s="96">
         <v>23190.87</v>
       </c>
-      <c r="BK56" t="s">
-        <v>114</v>
-      </c>
     </row>
-    <row r="57" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A57" s="241">
         <v>2554</v>
       </c>
@@ -13174,11 +12430,8 @@
       <c r="BJ57" s="96">
         <v>24211.27</v>
       </c>
-      <c r="BK57" t="s">
-        <v>115</v>
-      </c>
     </row>
-    <row r="58" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A58" s="241">
         <v>2554</v>
       </c>
@@ -13361,11 +12614,8 @@
       <c r="BJ58" s="96">
         <v>23996.240000000002</v>
       </c>
-      <c r="BK58" t="s">
-        <v>116</v>
-      </c>
     </row>
-    <row r="59" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A59" s="241">
         <v>2554</v>
       </c>
@@ -13548,11 +12798,8 @@
       <c r="BJ59" s="96">
         <v>24699.24</v>
       </c>
-      <c r="BK59" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="60" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A60" s="241">
         <v>2554</v>
       </c>
@@ -13735,11 +12982,8 @@
       <c r="BJ60" s="96">
         <v>23791.65</v>
       </c>
-      <c r="BK60" t="s">
-        <v>117</v>
-      </c>
     </row>
-    <row r="61" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A61" s="241">
         <v>2554</v>
       </c>
@@ -13922,11 +13166,8 @@
       <c r="BJ61" s="96">
         <v>22689.31</v>
       </c>
-      <c r="BK61" t="s">
-        <v>118</v>
-      </c>
     </row>
-    <row r="62" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A62" s="243">
         <v>2555</v>
       </c>
@@ -14113,11 +13354,8 @@
       <c r="BJ62" s="110">
         <v>17077.66</v>
       </c>
-      <c r="BK62" t="s">
-        <v>119</v>
-      </c>
     </row>
-    <row r="63" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A63" s="243">
         <v>2555</v>
       </c>
@@ -14304,11 +13542,8 @@
       <c r="BJ63" s="110">
         <v>20305.38</v>
       </c>
-      <c r="BK63" t="s">
-        <v>120</v>
-      </c>
     </row>
-    <row r="64" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A64" s="243">
         <v>2555</v>
       </c>
@@ -14495,11 +13730,8 @@
       <c r="BJ64" s="110">
         <v>22244.89</v>
       </c>
-      <c r="BK64" t="s">
-        <v>121</v>
-      </c>
     </row>
-    <row r="65" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A65" s="243">
         <v>2555</v>
       </c>
@@ -14686,11 +13918,8 @@
       <c r="BJ65" s="110">
         <v>17707.150000000001</v>
       </c>
-      <c r="BK65" t="s">
-        <v>122</v>
-      </c>
     </row>
-    <row r="66" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A66" s="243">
         <v>2555</v>
       </c>
@@ -14877,11 +14106,8 @@
       <c r="BJ66" s="110">
         <v>23475.77</v>
       </c>
-      <c r="BK66" t="s">
-        <v>123</v>
-      </c>
     </row>
-    <row r="67" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A67" s="243">
         <v>2555</v>
       </c>
@@ -15068,11 +14294,8 @@
       <c r="BJ67" s="110">
         <v>23084.38</v>
       </c>
-      <c r="BK67" t="s">
-        <v>124</v>
-      </c>
     </row>
-    <row r="68" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A68" s="243">
         <v>2555</v>
       </c>
@@ -15259,11 +14482,8 @@
       <c r="BJ68" s="110">
         <v>24169.5</v>
       </c>
-      <c r="BK68" t="s">
-        <v>125</v>
-      </c>
     </row>
-    <row r="69" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A69" s="243">
         <v>2555</v>
       </c>
@@ -15450,11 +14670,8 @@
       <c r="BJ69" s="110">
         <v>23388.67</v>
       </c>
-      <c r="BK69" t="s">
-        <v>126</v>
-      </c>
     </row>
-    <row r="70" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A70" s="243">
         <v>2555</v>
       </c>
@@ -15641,11 +14858,8 @@
       <c r="BJ70" s="110">
         <v>23321.55</v>
       </c>
-      <c r="BK70" t="s">
-        <v>127</v>
-      </c>
     </row>
-    <row r="71" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A71" s="243">
         <v>2555</v>
       </c>
@@ -15832,11 +15046,8 @@
       <c r="BJ71" s="110">
         <v>23708.3</v>
       </c>
-      <c r="BK71" t="s">
-        <v>128</v>
-      </c>
     </row>
-    <row r="72" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A72" s="243">
         <v>2555</v>
       </c>
@@ -16023,11 +15234,8 @@
       <c r="BJ72" s="110">
         <v>24621.98</v>
       </c>
-      <c r="BK72" t="s">
-        <v>128</v>
-      </c>
     </row>
-    <row r="73" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A73" s="243">
         <v>2555</v>
       </c>
@@ -16214,11 +15422,8 @@
       <c r="BJ73" s="110">
         <v>21313.31</v>
       </c>
-      <c r="BK73" t="s">
-        <v>129</v>
-      </c>
     </row>
-    <row r="74" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A74" s="245">
         <v>2556</v>
       </c>
@@ -16405,11 +15610,8 @@
       <c r="BJ74" s="127">
         <v>18907.599999999999</v>
       </c>
-      <c r="BK74" t="s">
-        <v>130</v>
-      </c>
     </row>
-    <row r="75" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A75" s="245">
         <v>2556</v>
       </c>
@@ -16596,11 +15798,8 @@
       <c r="BJ75" s="127">
         <v>17797.45</v>
       </c>
-      <c r="BK75" t="s">
-        <v>131</v>
-      </c>
     </row>
-    <row r="76" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A76" s="245">
         <v>2556</v>
       </c>
@@ -16787,11 +15986,8 @@
       <c r="BJ76" s="127">
         <v>19744.669999999998</v>
       </c>
-      <c r="BK76" t="s">
-        <v>132</v>
-      </c>
     </row>
-    <row r="77" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A77" s="245">
         <v>2556</v>
       </c>
@@ -16978,11 +16174,8 @@
       <c r="BJ77" s="127">
         <v>16578.63</v>
       </c>
-      <c r="BK77" t="s">
-        <v>133</v>
-      </c>
     </row>
-    <row r="78" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A78" s="245">
         <v>2556</v>
       </c>
@@ -17169,11 +16362,8 @@
       <c r="BJ78" s="127">
         <v>18744.78</v>
       </c>
-      <c r="BK78" t="s">
-        <v>134</v>
-      </c>
     </row>
-    <row r="79" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A79" s="245">
         <v>2556</v>
       </c>
@@ -17360,11 +16550,8 @@
       <c r="BJ79" s="127">
         <v>17906.89</v>
       </c>
-      <c r="BK79" t="s">
-        <v>135</v>
-      </c>
     </row>
-    <row r="80" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A80" s="245">
         <v>2556</v>
       </c>
@@ -17551,11 +16738,8 @@
       <c r="BJ80" s="135">
         <v>0</v>
       </c>
-      <c r="BK80" t="s">
-        <v>136</v>
-      </c>
     </row>
-    <row r="81" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A81" s="245">
         <v>2556</v>
       </c>
@@ -17742,11 +16926,8 @@
       <c r="BJ81" s="127">
         <v>19421.3</v>
       </c>
-      <c r="BK81" t="s">
-        <v>137</v>
-      </c>
     </row>
-    <row r="82" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A82" s="245">
         <v>2556</v>
       </c>
@@ -17933,11 +17114,8 @@
       <c r="BJ82" s="127">
         <v>19887.89</v>
       </c>
-      <c r="BK82" t="s">
-        <v>138</v>
-      </c>
     </row>
-    <row r="83" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A83" s="245">
         <v>2556</v>
       </c>
@@ -18124,11 +17302,8 @@
       <c r="BJ83" s="127">
         <v>21475.279999999999</v>
       </c>
-      <c r="BK83" t="s">
-        <v>139</v>
-      </c>
     </row>
-    <row r="84" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A84" s="245">
         <v>2556</v>
       </c>
@@ -18315,11 +17490,8 @@
       <c r="BJ84" s="127">
         <v>21441.81</v>
       </c>
-      <c r="BK84" t="s">
-        <v>140</v>
-      </c>
     </row>
-    <row r="85" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A85" s="245">
         <v>2556</v>
       </c>
@@ -18506,11 +17678,8 @@
       <c r="BJ85" s="143">
         <v>17442.05</v>
       </c>
-      <c r="BK85" t="s">
-        <v>141</v>
-      </c>
     </row>
-    <row r="86" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A86" s="247">
         <v>2557</v>
       </c>
@@ -18697,11 +17866,8 @@
       <c r="BJ86" s="154">
         <v>18100.84</v>
       </c>
-      <c r="BK86" t="s">
-        <v>142</v>
-      </c>
     </row>
-    <row r="87" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A87" s="247">
         <v>2557</v>
       </c>
@@ -18888,11 +18054,8 @@
       <c r="BJ87" s="154">
         <v>17085.73</v>
       </c>
-      <c r="BK87" t="s">
-        <v>143</v>
-      </c>
     </row>
-    <row r="88" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A88" s="247">
         <v>2557</v>
       </c>
@@ -19079,11 +18242,8 @@
       <c r="BJ88" s="154">
         <v>18957.07</v>
       </c>
-      <c r="BK88" t="s">
-        <v>144</v>
-      </c>
     </row>
-    <row r="89" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A89" s="247">
         <v>2557</v>
       </c>
@@ -19270,11 +18430,8 @@
       <c r="BJ89" s="154">
         <v>16913.61</v>
       </c>
-      <c r="BK89" t="s">
-        <v>145</v>
-      </c>
     </row>
-    <row r="90" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A90" s="247">
         <v>2557</v>
       </c>
@@ -19461,11 +18618,8 @@
       <c r="BJ90" s="154">
         <v>18141.39</v>
       </c>
-      <c r="BK90" t="s">
-        <v>146</v>
-      </c>
     </row>
-    <row r="91" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A91" s="247">
         <v>2557</v>
       </c>
@@ -19652,11 +18806,8 @@
       <c r="BJ91" s="154">
         <v>18427.490000000002</v>
       </c>
-      <c r="BK91" t="s">
-        <v>147</v>
-      </c>
     </row>
-    <row r="92" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A92" s="247">
         <v>2557</v>
       </c>
@@ -19843,11 +18994,8 @@
       <c r="BJ92" s="154">
         <v>19888.77</v>
       </c>
-      <c r="BK92" t="s">
-        <v>148</v>
-      </c>
     </row>
-    <row r="93" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A93" s="247">
         <v>2557</v>
       </c>
@@ -20034,11 +19182,8 @@
       <c r="BJ93" s="154">
         <v>18223.68</v>
       </c>
-      <c r="BK93" t="s">
-        <v>149</v>
-      </c>
     </row>
-    <row r="94" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A94" s="247">
         <v>2557</v>
       </c>
@@ -20225,11 +19370,8 @@
       <c r="BJ94" s="154">
         <v>19853.53</v>
       </c>
-      <c r="BK94" t="s">
-        <v>150</v>
-      </c>
     </row>
-    <row r="95" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A95" s="247">
         <v>2557</v>
       </c>
@@ -20416,11 +19558,8 @@
       <c r="BJ95" s="154">
         <v>23204.77</v>
       </c>
-      <c r="BK95" t="s">
-        <v>151</v>
-      </c>
     </row>
-    <row r="96" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A96" s="247">
         <v>2557</v>
       </c>
@@ -20607,11 +19746,8 @@
       <c r="BJ96" s="154">
         <v>20410.349999999999</v>
       </c>
-      <c r="BK96" t="s">
-        <v>65</v>
-      </c>
     </row>
-    <row r="97" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A97" s="247">
         <v>2557</v>
       </c>
@@ -20798,11 +19934,8 @@
       <c r="BJ97" s="154">
         <v>18653.27</v>
       </c>
-      <c r="BK97" t="s">
-        <v>66</v>
-      </c>
     </row>
-    <row r="98" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A98" s="249">
         <v>2558</v>
       </c>
@@ -20989,11 +20122,8 @@
       <c r="BJ98" s="165">
         <v>16893.82</v>
       </c>
-      <c r="BK98" t="s">
-        <v>152</v>
-      </c>
     </row>
-    <row r="99" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A99" s="249">
         <v>2558</v>
       </c>
@@ -21180,11 +20310,8 @@
       <c r="BJ99" s="165">
         <v>14994.79</v>
       </c>
-      <c r="BK99" t="s">
-        <v>99</v>
-      </c>
     </row>
-    <row r="100" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A100" s="249">
         <v>2558</v>
       </c>
@@ -21371,11 +20498,8 @@
       <c r="BJ100" s="165">
         <v>17304.37</v>
       </c>
-      <c r="BK100" t="s">
-        <v>101</v>
-      </c>
     </row>
-    <row r="101" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A101" s="249">
         <v>2558</v>
       </c>
@@ -21562,11 +20686,8 @@
       <c r="BJ101" s="165">
         <v>15311.86</v>
       </c>
-      <c r="BK101" t="s">
-        <v>142</v>
-      </c>
     </row>
-    <row r="102" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A102" s="249">
         <v>2558</v>
       </c>
@@ -21753,11 +20874,8 @@
       <c r="BJ102" s="165">
         <v>16320.06</v>
       </c>
-      <c r="BK102" t="s">
-        <v>153</v>
-      </c>
     </row>
-    <row r="103" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A103" s="249">
         <v>2558</v>
       </c>
@@ -21944,11 +21062,8 @@
       <c r="BJ103" s="165">
         <v>16867.64</v>
       </c>
-      <c r="BK103" t="s">
-        <v>154</v>
-      </c>
     </row>
-    <row r="104" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A104" s="249">
         <v>2558</v>
       </c>
@@ -22135,11 +21250,8 @@
       <c r="BJ104" s="165">
         <v>17145.830000000002</v>
       </c>
-      <c r="BK104" t="s">
-        <v>155</v>
-      </c>
     </row>
-    <row r="105" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A105" s="249">
         <v>2558</v>
       </c>
@@ -22326,11 +21438,8 @@
       <c r="BJ105" s="165">
         <v>17100.71</v>
       </c>
-      <c r="BK105" t="s">
-        <v>156</v>
-      </c>
     </row>
-    <row r="106" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A106" s="249">
         <v>2558</v>
       </c>
@@ -22517,11 +21626,8 @@
       <c r="BJ106" s="165">
         <v>18848.080000000002</v>
       </c>
-      <c r="BK106" t="s">
-        <v>157</v>
-      </c>
     </row>
-    <row r="107" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A107" s="249">
         <v>2558</v>
       </c>
@@ -22708,11 +21814,8 @@
       <c r="BJ107" s="165">
         <v>19390.88</v>
       </c>
-      <c r="BK107" t="s">
-        <v>158</v>
-      </c>
     </row>
-    <row r="108" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A108" s="249">
         <v>2558</v>
       </c>
@@ -22899,11 +22002,8 @@
       <c r="BJ108" s="165">
         <v>18920.3</v>
       </c>
-      <c r="BK108" t="s">
-        <v>159</v>
-      </c>
     </row>
-    <row r="109" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A109" s="249">
         <v>2558</v>
       </c>
@@ -23090,11 +22190,8 @@
       <c r="BJ109" s="165">
         <v>19050.240000000002</v>
       </c>
-      <c r="BK109" t="s">
-        <v>160</v>
-      </c>
     </row>
-    <row r="110" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A110" s="251">
         <v>2559</v>
       </c>
@@ -23281,11 +22378,8 @@
       <c r="BJ110" s="176">
         <v>15205.95</v>
       </c>
-      <c r="BK110" t="s">
-        <v>161</v>
-      </c>
     </row>
-    <row r="111" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A111" s="251">
         <v>2559</v>
       </c>
@@ -23472,11 +22566,8 @@
       <c r="BJ111" s="176">
         <v>16133.29</v>
       </c>
-      <c r="BK111" t="s">
-        <v>162</v>
-      </c>
     </row>
-    <row r="112" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A112" s="251">
         <v>2559</v>
       </c>
@@ -23663,11 +22754,8 @@
       <c r="BJ112" s="176">
         <v>18536.59</v>
       </c>
-      <c r="BK112" t="s">
-        <v>163</v>
-      </c>
     </row>
-    <row r="113" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A113" s="251">
         <v>2559</v>
       </c>
@@ -23854,11 +22942,8 @@
       <c r="BJ113" s="176">
         <v>15298.45</v>
       </c>
-      <c r="BK113" t="s">
-        <v>164</v>
-      </c>
     </row>
-    <row r="114" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A114" s="251">
         <v>2559</v>
       </c>
@@ -24045,11 +23130,8 @@
       <c r="BJ114" s="176">
         <v>18775.150000000001</v>
       </c>
-      <c r="BK114" t="s">
-        <v>165</v>
-      </c>
     </row>
-    <row r="115" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A115" s="251">
         <v>2559</v>
       </c>
@@ -24236,11 +23318,8 @@
       <c r="BJ115" s="176">
         <v>19300.98</v>
       </c>
-      <c r="BK115" t="s">
-        <v>163</v>
-      </c>
     </row>
-    <row r="116" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A116" s="251">
         <v>2559</v>
       </c>
@@ -24427,11 +23506,8 @@
       <c r="BJ116" s="176">
         <v>18347.43</v>
       </c>
-      <c r="BK116" t="s">
-        <v>166</v>
-      </c>
     </row>
-    <row r="117" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A117" s="251">
         <v>2559</v>
       </c>
@@ -24618,11 +23694,8 @@
       <c r="BJ117" s="176">
         <v>18225.93</v>
       </c>
-      <c r="BK117" t="s">
-        <v>167</v>
-      </c>
     </row>
-    <row r="118" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A118" s="251">
         <v>2559</v>
       </c>
@@ -24809,11 +23882,8 @@
       <c r="BJ118" s="176">
         <v>20374.34</v>
       </c>
-      <c r="BK118" t="s">
-        <v>168</v>
-      </c>
     </row>
-    <row r="119" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A119" s="251">
         <v>2559</v>
       </c>
@@ -25000,11 +24070,8 @@
       <c r="BJ119" s="176">
         <v>20510.2</v>
       </c>
-      <c r="BK119" t="s">
-        <v>169</v>
-      </c>
     </row>
-    <row r="120" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A120" s="251">
         <v>2559</v>
       </c>
@@ -25191,11 +24258,8 @@
       <c r="BJ120" s="176">
         <v>20712.71</v>
       </c>
-      <c r="BK120" t="s">
-        <v>170</v>
-      </c>
     </row>
-    <row r="121" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A121" s="251">
         <v>2559</v>
       </c>
@@ -25382,11 +24446,8 @@
       <c r="BJ121" s="176">
         <v>19125.77</v>
       </c>
-      <c r="BK121" t="s">
-        <v>171</v>
-      </c>
     </row>
-    <row r="122" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A122" s="235">
         <v>2560</v>
       </c>
@@ -25561,11 +24622,8 @@
       <c r="BJ122" s="58">
         <v>15228.71</v>
       </c>
-      <c r="BK122" t="s">
-        <v>172</v>
-      </c>
     </row>
-    <row r="123" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A123" s="235">
         <v>2560</v>
       </c>
@@ -25740,11 +24798,8 @@
       <c r="BJ123" s="58">
         <v>16020.52</v>
       </c>
-      <c r="BK123" t="s">
-        <v>173</v>
-      </c>
     </row>
-    <row r="124" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A124" s="235">
         <v>2560</v>
       </c>
@@ -25919,11 +24974,8 @@
       <c r="BJ124" s="58">
         <v>19017.93</v>
       </c>
-      <c r="BK124" t="s">
-        <v>174</v>
-      </c>
     </row>
-    <row r="125" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A125" s="235">
         <v>2560</v>
       </c>
@@ -26098,11 +25150,8 @@
       <c r="BJ125" s="58">
         <v>13477.68</v>
       </c>
-      <c r="BK125" t="s">
-        <v>168</v>
-      </c>
     </row>
-    <row r="126" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A126" s="235">
         <v>2560</v>
       </c>
@@ -26277,11 +25326,8 @@
       <c r="BJ126" s="58">
         <v>19850.189999999999</v>
       </c>
-      <c r="BK126" t="s">
-        <v>175</v>
-      </c>
     </row>
-    <row r="127" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A127" s="235">
         <v>2560</v>
       </c>
@@ -26456,11 +25502,8 @@
       <c r="BJ127" s="58">
         <v>19722.21</v>
       </c>
-      <c r="BK127" t="s">
-        <v>176</v>
-      </c>
     </row>
-    <row r="128" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A128" s="235">
         <v>2560</v>
       </c>
@@ -26635,11 +25678,8 @@
       <c r="BJ128" s="58">
         <v>18191.5</v>
       </c>
-      <c r="BK128" t="s">
-        <v>177</v>
-      </c>
     </row>
-    <row r="129" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A129" s="235">
         <v>2560</v>
       </c>
@@ -26814,11 +25854,8 @@
       <c r="BJ129" s="58">
         <v>19875.2</v>
       </c>
-      <c r="BK129" t="s">
-        <v>178</v>
-      </c>
     </row>
-    <row r="130" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A130" s="235">
         <v>2560</v>
       </c>
@@ -26993,11 +26030,8 @@
       <c r="BJ130" s="58">
         <v>19466.73</v>
       </c>
-      <c r="BK130" t="s">
-        <v>179</v>
-      </c>
     </row>
-    <row r="131" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A131" s="235">
         <v>2560</v>
       </c>
@@ -27172,11 +26206,8 @@
       <c r="BJ131" s="58">
         <v>19459.77</v>
       </c>
-      <c r="BK131" t="s">
-        <v>180</v>
-      </c>
     </row>
-    <row r="132" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A132" s="235">
         <v>2560</v>
       </c>
@@ -27351,11 +26382,8 @@
       <c r="BJ132" s="58">
         <v>20141.7</v>
       </c>
-      <c r="BK132" t="s">
-        <v>181</v>
-      </c>
     </row>
-    <row r="133" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A133" s="235">
         <v>2560</v>
       </c>
@@ -27530,11 +26558,8 @@
       <c r="BJ133" s="58">
         <v>17995.490000000002</v>
       </c>
-      <c r="BK133" t="s">
-        <v>182</v>
-      </c>
     </row>
-    <row r="134" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A134" s="239">
         <v>2561</v>
       </c>
@@ -27713,11 +26738,8 @@
       <c r="BJ134" s="83">
         <v>17166.28</v>
       </c>
-      <c r="BK134" t="s">
-        <v>136</v>
-      </c>
     </row>
-    <row r="135" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A135" s="239">
         <v>2561</v>
       </c>
@@ -27896,11 +26918,8 @@
       <c r="BJ135" s="83">
         <v>14811.55</v>
       </c>
-      <c r="BK135" t="s">
-        <v>183</v>
-      </c>
     </row>
-    <row r="136" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A136" s="239">
         <v>2561</v>
       </c>
@@ -28079,11 +27098,8 @@
       <c r="BJ136" s="83">
         <v>17629.91</v>
       </c>
-      <c r="BK136" t="s">
-        <v>116</v>
-      </c>
     </row>
-    <row r="137" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A137" s="239">
         <v>2561</v>
       </c>
@@ -28262,11 +27278,8 @@
       <c r="BJ137" s="83">
         <v>14777.07</v>
       </c>
-      <c r="BK137" t="s">
-        <v>124</v>
-      </c>
     </row>
-    <row r="138" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A138" s="239">
         <v>2561</v>
       </c>
@@ -28445,11 +27458,8 @@
       <c r="BJ138" s="83">
         <v>18078.12</v>
       </c>
-      <c r="BK138" t="s">
-        <v>184</v>
-      </c>
     </row>
-    <row r="139" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A139" s="239">
         <v>2561</v>
       </c>
@@ -28628,11 +27638,8 @@
       <c r="BJ139" s="83">
         <v>17604.05</v>
       </c>
-      <c r="BK139" t="s">
-        <v>185</v>
-      </c>
     </row>
-    <row r="140" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A140" s="239">
         <v>2561</v>
       </c>
@@ -28811,11 +27818,8 @@
       <c r="BJ140" s="83">
         <v>17906.900000000001</v>
       </c>
-      <c r="BK140" t="s">
-        <v>186</v>
-      </c>
     </row>
-    <row r="141" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A141" s="239">
         <v>2561</v>
       </c>
@@ -28994,11 +27998,8 @@
       <c r="BJ141" s="83">
         <v>19512.52</v>
       </c>
-      <c r="BK141" t="s">
-        <v>187</v>
-      </c>
     </row>
-    <row r="142" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A142" s="239">
         <v>2561</v>
       </c>
@@ -29177,11 +28178,8 @@
       <c r="BJ142" s="83">
         <v>18046.12</v>
       </c>
-      <c r="BK142" t="s">
-        <v>188</v>
-      </c>
     </row>
-    <row r="143" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A143" s="239">
         <v>2561</v>
       </c>
@@ -29360,11 +28358,8 @@
       <c r="BJ143" s="83">
         <v>19866.91</v>
       </c>
-      <c r="BK143" t="s">
-        <v>189</v>
-      </c>
     </row>
-    <row r="144" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A144" s="239">
         <v>2561</v>
       </c>
@@ -29543,11 +28538,8 @@
       <c r="BJ144" s="83">
         <v>19988.79</v>
       </c>
-      <c r="BK144" t="s">
-        <v>190</v>
-      </c>
     </row>
-    <row r="145" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A145" s="239">
         <v>2561</v>
       </c>
@@ -29726,11 +28718,8 @@
       <c r="BJ145" s="83">
         <v>17648.37</v>
       </c>
-      <c r="BK145" t="s">
-        <v>191</v>
-      </c>
     </row>
-    <row r="146" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A146" s="243">
         <v>2562</v>
       </c>
@@ -29909,11 +28898,8 @@
       <c r="BJ146" s="110">
         <v>16289.75</v>
       </c>
-      <c r="BK146" t="s">
-        <v>192</v>
-      </c>
     </row>
-    <row r="147" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A147" s="243">
         <v>2562</v>
       </c>
@@ -30092,11 +29078,8 @@
       <c r="BJ147" s="110">
         <v>15071.12</v>
       </c>
-      <c r="BK147" t="s">
-        <v>193</v>
-      </c>
     </row>
-    <row r="148" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A148" s="243">
         <v>2562</v>
       </c>
@@ -30275,11 +29258,8 @@
       <c r="BJ148" s="110">
         <v>16802.86</v>
       </c>
-      <c r="BK148" t="s">
-        <v>194</v>
-      </c>
     </row>
-    <row r="149" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A149" s="243">
         <v>2562</v>
       </c>
@@ -30458,11 +29438,8 @@
       <c r="BJ149" s="110">
         <v>15175.4</v>
       </c>
-      <c r="BK149" t="s">
-        <v>195</v>
-      </c>
     </row>
-    <row r="150" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A150" s="243">
         <v>2562</v>
       </c>
@@ -30641,11 +29618,8 @@
       <c r="BJ150" s="110">
         <v>17662.03</v>
       </c>
-      <c r="BK150" t="s">
-        <v>118</v>
-      </c>
     </row>
-    <row r="151" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A151" s="243">
         <v>2562</v>
       </c>
@@ -30824,11 +29798,8 @@
       <c r="BJ151" s="110">
         <v>16080.92</v>
       </c>
-      <c r="BK151" t="s">
-        <v>196</v>
-      </c>
     </row>
-    <row r="152" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A152" s="243">
         <v>2562</v>
       </c>
@@ -31007,11 +29978,8 @@
       <c r="BJ152" s="110">
         <v>16607.72</v>
       </c>
-      <c r="BK152" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="153" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A153" s="243">
         <v>2562</v>
       </c>
@@ -31190,11 +30158,8 @@
       <c r="BJ153" s="110">
         <v>16471.13</v>
       </c>
-      <c r="BK153" t="s">
-        <v>197</v>
-      </c>
     </row>
-    <row r="154" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A154" s="243">
         <v>2562</v>
       </c>
@@ -31373,11 +30338,8 @@
       <c r="BJ154" s="110">
         <v>16963.400000000001</v>
       </c>
-      <c r="BK154" t="s">
-        <v>198</v>
-      </c>
     </row>
-    <row r="155" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A155" s="243">
         <v>2562</v>
       </c>
@@ -31556,11 +30518,8 @@
       <c r="BJ155" s="110">
         <v>18595.740000000002</v>
       </c>
-      <c r="BK155" t="s">
-        <v>199</v>
-      </c>
     </row>
-    <row r="156" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A156" s="243">
         <v>2562</v>
       </c>
@@ -31739,11 +30698,8 @@
       <c r="BJ156" s="110">
         <v>17162.22</v>
       </c>
-      <c r="BK156" t="s">
-        <v>200</v>
-      </c>
     </row>
-    <row r="157" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A157" s="243">
         <v>2562</v>
       </c>
@@ -31922,11 +30878,8 @@
       <c r="BJ157" s="110">
         <v>14700.88</v>
       </c>
-      <c r="BK157" t="s">
-        <v>131</v>
-      </c>
     </row>
-    <row r="158" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A158" s="253">
         <v>2563</v>
       </c>
@@ -32105,11 +31058,8 @@
       <c r="BJ158" s="127">
         <v>13364</v>
       </c>
-      <c r="BK158" t="s">
-        <v>192</v>
-      </c>
     </row>
-    <row r="159" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A159" s="253">
         <v>2563</v>
       </c>
@@ -32288,11 +31238,8 @@
       <c r="BJ159" s="127">
         <v>14814.27</v>
       </c>
-      <c r="BK159" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="160" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A160" s="253">
         <v>2563</v>
       </c>
@@ -32471,11 +31418,8 @@
       <c r="BJ160" s="127">
         <v>16252.57</v>
       </c>
-      <c r="BK160" t="s">
-        <v>202</v>
-      </c>
     </row>
-    <row r="161" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A161" s="253">
         <v>2563</v>
       </c>
@@ -32654,11 +31598,8 @@
       <c r="BJ161" s="127">
         <v>17642.599999999999</v>
       </c>
-      <c r="BK161" t="s">
-        <v>203</v>
-      </c>
     </row>
-    <row r="162" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A162" s="253">
         <v>2563</v>
       </c>
@@ -32837,11 +31778,8 @@
       <c r="BJ162" s="127">
         <v>17801.13</v>
       </c>
-      <c r="BK162" t="s">
-        <v>204</v>
-      </c>
     </row>
-    <row r="163" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A163" s="253">
         <v>2563</v>
       </c>
@@ -33020,11 +31958,8 @@
       <c r="BJ163" s="127">
         <v>17647.41</v>
       </c>
-      <c r="BK163" t="s">
-        <v>205</v>
-      </c>
     </row>
-    <row r="164" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A164" s="253">
         <v>2563</v>
       </c>
@@ -33203,11 +32138,8 @@
       <c r="BJ164" s="127">
         <v>16544.27</v>
       </c>
-      <c r="BK164" t="s">
-        <v>206</v>
-      </c>
     </row>
-    <row r="165" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A165" s="253">
         <v>2563</v>
       </c>
@@ -33386,11 +32318,8 @@
       <c r="BJ165" s="127">
         <v>16687.810000000001</v>
       </c>
-      <c r="BK165" t="s">
-        <v>207</v>
-      </c>
     </row>
-    <row r="166" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A166" s="253">
         <v>2563</v>
       </c>
@@ -33569,11 +32498,8 @@
       <c r="BJ166" s="127">
         <v>17062.88</v>
       </c>
-      <c r="BK166" t="s">
-        <v>208</v>
-      </c>
     </row>
-    <row r="167" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A167" s="253">
         <v>2563</v>
       </c>
@@ -33752,11 +32678,8 @@
       <c r="BJ167" s="127">
         <v>17901.79</v>
       </c>
-      <c r="BK167" t="s">
-        <v>139</v>
-      </c>
     </row>
-    <row r="168" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A168" s="253">
         <v>2563</v>
       </c>
@@ -33935,11 +32858,8 @@
       <c r="BJ168" s="127">
         <v>16373.64</v>
       </c>
-      <c r="BK168" t="s">
-        <v>209</v>
-      </c>
     </row>
-    <row r="169" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A169" s="253">
         <v>2563</v>
       </c>
@@ -34118,11 +33038,8 @@
       <c r="BJ169" s="127">
         <v>14693.26</v>
       </c>
-      <c r="BK169" t="s">
-        <v>210</v>
-      </c>
     </row>
-    <row r="170" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A170" s="255">
         <v>2564</v>
       </c>
@@ -34301,11 +33218,8 @@
       <c r="BJ170" s="165">
         <v>13186.45</v>
       </c>
-      <c r="BK170" t="s">
-        <v>211</v>
-      </c>
     </row>
-    <row r="171" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A171" s="255">
         <v>2564</v>
       </c>
@@ -34484,11 +33398,8 @@
       <c r="BJ171" s="165">
         <v>13317.76</v>
       </c>
-      <c r="BK171" t="s">
-        <v>212</v>
-      </c>
     </row>
-    <row r="172" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A172" s="255">
         <v>2564</v>
       </c>
@@ -34667,11 +33578,8 @@
       <c r="BJ172" s="165">
         <v>16536.53</v>
       </c>
-      <c r="BK172" t="s">
-        <v>213</v>
-      </c>
     </row>
-    <row r="173" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A173" s="255">
         <v>2564</v>
       </c>
@@ -34850,11 +33758,8 @@
       <c r="BJ173" s="165">
         <v>14891.98</v>
       </c>
-      <c r="BK173" t="s">
-        <v>139</v>
-      </c>
     </row>
-    <row r="174" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A174" s="255">
         <v>2564</v>
       </c>
@@ -35033,11 +33938,8 @@
       <c r="BJ174" s="165">
         <v>14870.49</v>
       </c>
-      <c r="BK174" t="s">
-        <v>214</v>
-      </c>
     </row>
-    <row r="175" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A175" s="255">
         <v>2564</v>
       </c>
@@ -35216,11 +34118,8 @@
       <c r="BJ175" s="165">
         <v>17446.96</v>
       </c>
-      <c r="BK175" t="s">
-        <v>215</v>
-      </c>
     </row>
-    <row r="176" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A176" s="255">
         <v>2564</v>
       </c>
@@ -35399,11 +34298,8 @@
       <c r="BJ176" s="165">
         <v>15894.17</v>
       </c>
-      <c r="BK176" t="s">
-        <v>216</v>
-      </c>
     </row>
-    <row r="177" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A177" s="255">
         <v>2564</v>
       </c>
@@ -35582,11 +34478,8 @@
       <c r="BJ177" s="165">
         <v>16024.79</v>
       </c>
-      <c r="BK177" t="s">
-        <v>217</v>
-      </c>
     </row>
-    <row r="178" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A178" s="255">
         <v>2564</v>
       </c>
@@ -35765,11 +34658,8 @@
       <c r="BJ178" s="165">
         <v>17563.68</v>
       </c>
-      <c r="BK178" t="s">
-        <v>218</v>
-      </c>
     </row>
-    <row r="179" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A179" s="255">
         <v>2564</v>
       </c>
@@ -35948,11 +34838,8 @@
       <c r="BJ179" s="165">
         <v>18628.79</v>
       </c>
-      <c r="BK179" t="s">
-        <v>177</v>
-      </c>
     </row>
-    <row r="180" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A180" s="255">
         <v>2564</v>
       </c>
@@ -36131,11 +35018,8 @@
       <c r="BJ180" s="165">
         <v>18670.96</v>
       </c>
-      <c r="BK180" t="s">
-        <v>219</v>
-      </c>
     </row>
-    <row r="181" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A181" s="255">
         <v>2564</v>
       </c>
@@ -36314,11 +35198,8 @@
       <c r="BJ181" s="165">
         <v>18186.98</v>
       </c>
-      <c r="BK181" t="s">
-        <v>220</v>
-      </c>
     </row>
-    <row r="182" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A182" s="237">
         <v>2565</v>
       </c>
@@ -36497,11 +35378,8 @@
       <c r="BJ182" s="71">
         <v>15984.2</v>
       </c>
-      <c r="BK182" t="s">
-        <v>180</v>
-      </c>
     </row>
-    <row r="183" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A183" s="237">
         <v>2565</v>
       </c>
@@ -36680,11 +35558,8 @@
       <c r="BJ183" s="71">
         <v>17619.38</v>
       </c>
-      <c r="BK183" t="s">
-        <v>221</v>
-      </c>
     </row>
-    <row r="184" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A184" s="237">
         <v>2565</v>
       </c>
@@ -36863,11 +35738,8 @@
       <c r="BJ184" s="71">
         <v>19233.55</v>
       </c>
-      <c r="BK184" t="s">
-        <v>222</v>
-      </c>
     </row>
-    <row r="185" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A185" s="237">
         <v>2565</v>
       </c>
@@ -37046,11 +35918,8 @@
       <c r="BJ185" s="71">
         <v>17366.38</v>
       </c>
-      <c r="BK185" t="s">
-        <v>223</v>
-      </c>
     </row>
-    <row r="186" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A186" s="237">
         <v>2565</v>
       </c>
@@ -37229,11 +36098,8 @@
       <c r="BJ186" s="71">
         <v>18732</v>
       </c>
-      <c r="BK186" t="s">
-        <v>224</v>
-      </c>
     </row>
-    <row r="187" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A187" s="237">
         <v>2565</v>
       </c>
@@ -37412,11 +36278,8 @@
       <c r="BJ187" s="71">
         <v>19982.939999999999</v>
       </c>
-      <c r="BK187" t="s">
-        <v>225</v>
-      </c>
     </row>
-    <row r="188" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A188" s="237">
         <v>2565</v>
       </c>
@@ -37595,11 +36458,8 @@
       <c r="BJ188" s="71">
         <v>19448.78</v>
       </c>
-      <c r="BK188" t="s">
-        <v>226</v>
-      </c>
     </row>
-    <row r="189" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A189" s="237">
         <v>2565</v>
       </c>
@@ -37778,11 +36638,8 @@
       <c r="BJ189" s="71">
         <v>20503.32</v>
       </c>
-      <c r="BK189" t="s">
-        <v>227</v>
-      </c>
     </row>
-    <row r="190" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A190" s="237">
         <v>2565</v>
       </c>
@@ -37961,11 +36818,8 @@
       <c r="BJ190" s="71">
         <v>21304.65</v>
       </c>
-      <c r="BK190" t="s">
-        <v>228</v>
-      </c>
     </row>
-    <row r="191" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A191" s="237">
         <v>2565</v>
       </c>
@@ -38144,11 +36998,8 @@
       <c r="BJ191" s="71">
         <v>19590.810000000001</v>
       </c>
-      <c r="BK191" t="s">
-        <v>229</v>
-      </c>
     </row>
-    <row r="192" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A192" s="237">
         <v>2565</v>
       </c>
@@ -38327,11 +37178,8 @@
       <c r="BJ192" s="71">
         <v>20400.349999999999</v>
       </c>
-      <c r="BK192" t="s">
-        <v>230</v>
-      </c>
     </row>
-    <row r="193" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A193" s="237">
         <v>2565</v>
       </c>
@@ -38510,11 +37358,8 @@
       <c r="BJ193" s="71">
         <v>18917.96</v>
       </c>
-      <c r="BK193" t="s">
-        <v>231</v>
-      </c>
     </row>
-    <row r="194" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A194" s="256">
         <v>2566</v>
       </c>
@@ -38697,11 +37542,8 @@
       <c r="BJ194" s="213">
         <v>14231.17</v>
       </c>
-      <c r="BK194" t="s">
-        <v>232</v>
-      </c>
     </row>
-    <row r="195" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A195" s="256">
         <v>2566</v>
       </c>
@@ -38884,11 +37726,8 @@
       <c r="BJ195" s="213">
         <v>15790.87</v>
       </c>
-      <c r="BK195" t="s">
-        <v>233</v>
-      </c>
     </row>
-    <row r="196" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A196" s="256">
         <v>2566</v>
       </c>
@@ -39071,11 +37910,8 @@
       <c r="BJ196" s="213">
         <v>18347.82</v>
       </c>
-      <c r="BK196" t="s">
-        <v>234</v>
-      </c>
     </row>
-    <row r="197" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A197" s="256">
         <v>2566</v>
       </c>
@@ -39258,11 +38094,8 @@
       <c r="BJ197" s="213">
         <v>15005.84</v>
       </c>
-      <c r="BK197" t="s">
-        <v>235</v>
-      </c>
     </row>
-    <row r="198" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A198" s="256">
         <v>2566</v>
       </c>
@@ -39445,11 +38278,8 @@
       <c r="BJ198" s="213">
         <v>18600.18</v>
       </c>
-      <c r="BK198" t="s">
-        <v>236</v>
-      </c>
     </row>
-    <row r="199" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A199" s="256">
         <v>2566</v>
       </c>
@@ -39632,11 +38462,8 @@
       <c r="BJ199" s="213">
         <v>17836.32</v>
       </c>
-      <c r="BK199" t="s">
-        <v>237</v>
-      </c>
     </row>
-    <row r="200" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A200" s="256">
         <v>2566</v>
       </c>
@@ -39819,11 +38646,8 @@
       <c r="BJ200" s="213">
         <v>17644.12</v>
       </c>
-      <c r="BK200" t="s">
-        <v>238</v>
-      </c>
     </row>
-    <row r="201" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A201" s="256">
         <v>2566</v>
       </c>
@@ -40006,11 +38830,8 @@
       <c r="BJ201" s="213">
         <v>17943.28</v>
       </c>
-      <c r="BK201" t="s">
-        <v>239</v>
-      </c>
     </row>
-    <row r="202" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A202" s="256">
         <v>2566</v>
       </c>
@@ -40193,11 +39014,8 @@
       <c r="BJ202" s="213">
         <v>18910.919999999998</v>
       </c>
-      <c r="BK202" t="s">
-        <v>240</v>
-      </c>
     </row>
-    <row r="203" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A203" s="256">
         <v>2566</v>
       </c>
@@ -40380,11 +39198,8 @@
       <c r="BJ203" s="213">
         <v>19164.41</v>
       </c>
-      <c r="BK203" t="s">
-        <v>241</v>
-      </c>
     </row>
-    <row r="204" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A204" s="256">
         <v>2566</v>
       </c>
@@ -40567,11 +39382,8 @@
       <c r="BJ204" s="213">
         <v>20329.53</v>
       </c>
-      <c r="BK204" t="s">
-        <v>242</v>
-      </c>
     </row>
-    <row r="205" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A205" s="256">
         <v>2566</v>
       </c>
@@ -40754,11 +39566,8 @@
       <c r="BJ205" s="213">
         <v>17481.09</v>
       </c>
-      <c r="BK205" t="s">
-        <v>243</v>
-      </c>
     </row>
-    <row r="206" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A206" s="243">
         <v>2567</v>
       </c>
@@ -40937,11 +39746,8 @@
       <c r="BJ206" s="110">
         <v>17136.61</v>
       </c>
-      <c r="BK206" t="s">
-        <v>244</v>
-      </c>
     </row>
-    <row r="207" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A207" s="243">
         <v>2567</v>
       </c>
@@ -41120,11 +39926,8 @@
       <c r="BJ207" s="110">
         <v>19243.61</v>
       </c>
-      <c r="BK207" t="s">
-        <v>245</v>
-      </c>
     </row>
-    <row r="208" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A208" s="243">
         <v>2567</v>
       </c>
@@ -41303,11 +40106,8 @@
       <c r="BJ208" s="110">
         <v>21220.400000000001</v>
       </c>
-      <c r="BK208" t="s">
-        <v>246</v>
-      </c>
     </row>
-    <row r="209" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A209" s="243">
         <v>2567</v>
       </c>
@@ -41486,11 +40286,8 @@
       <c r="BJ209" s="110">
         <v>18506.32</v>
       </c>
-      <c r="BK209" t="s">
-        <v>247</v>
-      </c>
     </row>
-    <row r="210" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A210" s="243">
         <v>2567</v>
       </c>
@@ -41669,11 +40466,8 @@
       <c r="BJ210" s="110">
         <v>20788.13</v>
       </c>
-      <c r="BK210" t="s">
-        <v>248</v>
-      </c>
     </row>
-    <row r="211" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A211" s="243">
         <v>2567</v>
       </c>
@@ -41852,11 +40646,8 @@
       <c r="BJ211" s="110">
         <v>18684.82</v>
       </c>
-      <c r="BK211" t="s">
-        <v>249</v>
-      </c>
     </row>
-    <row r="212" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A212" s="243">
         <v>2567</v>
       </c>
@@ -42035,11 +40826,8 @@
       <c r="BJ212" s="110">
         <v>21648.31</v>
       </c>
-      <c r="BK212" t="s">
-        <v>244</v>
-      </c>
     </row>
-    <row r="213" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A213" s="243">
         <v>2567</v>
       </c>
@@ -42218,11 +41006,8 @@
       <c r="BJ213" s="110">
         <v>22361.02</v>
       </c>
-      <c r="BK213" t="s">
-        <v>176</v>
-      </c>
     </row>
-    <row r="214" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A214" s="243">
         <v>2567</v>
       </c>
@@ -42401,11 +41186,8 @@
       <c r="BJ214" s="110">
         <v>20545.61</v>
       </c>
-      <c r="BK214" t="s">
-        <v>144</v>
-      </c>
     </row>
-    <row r="215" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A215" s="243">
         <v>2567</v>
       </c>
@@ -42584,11 +41366,8 @@
       <c r="BJ215" s="110">
         <v>20527.189999999999</v>
       </c>
-      <c r="BK215" t="s">
-        <v>154</v>
-      </c>
     </row>
-    <row r="216" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A216" s="243">
         <v>2567</v>
       </c>
@@ -42767,11 +41546,8 @@
       <c r="BJ216" s="110">
         <v>19657.150000000001</v>
       </c>
-      <c r="BK216" t="s">
-        <v>250</v>
-      </c>
     </row>
-    <row r="217" spans="1:63" ht="21" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:62" ht="21" x14ac:dyDescent="0.3">
       <c r="A217" s="243">
         <v>2567</v>
       </c>
@@ -42950,9 +41726,6 @@
       <c r="BJ217" s="229">
         <v>19742.45</v>
       </c>
-      <c r="BK217" t="s">
-        <v>251</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>